<commit_message>
refactored colormap setting, added self.cluster_info, added methods for editing self.cluster_info, added method for defining each clusters colour
</commit_message>
<xml_diff>
--- a/Example data/test_output/NW13-33/clustering_stats.xlsx
+++ b/Example data/test_output/NW13-33/clustering_stats.xlsx
@@ -496,62 +496,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>43.851741655185236</t>
+          <t>125.28370650382863</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>64.27768432975226</t>
+          <t>14.377823010565086</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.239850558293254</t>
+          <t>7.934089367064069</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>139.10319761298993</t>
+          <t>191.31520790927595</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12.489878029195228</t>
+          <t>3.110497237569061</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.9125664584513173</t>
+          <t>1.576427255985267</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>7.885585806418893</t>
+          <t>7.980905301928855</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.2620470470893523</t>
+          <t>0.4554618590675584</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.1254194595417009</t>
+          <t>0.5097412038383251</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.5101135182195474</t>
+          <t>0.3293593098769022</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>144.39584301858724</t>
+          <t>43.41106910923718</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>16.418445231474045</t>
+          <t>58.056120965396914</t>
         </is>
       </c>
     </row>
@@ -563,47 +563,47 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>117.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>142.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>6.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>160.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>18.0</t>
         </is>
       </c>
     </row>
@@ -630,62 +630,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>29.985004965492266</t>
+          <t>39.1210479345314</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25.708437564918547</t>
+          <t>15.303125164767756</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.357641118752377</t>
+          <t>5.915196477056346</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>204.70617457675593</t>
+          <t>152.99240017839574</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>17.616434600303133</t>
+          <t>6.067358272016304</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1.2782468645916572</t>
+          <t>1.6308248578071178</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>6.237274425561211</t>
+          <t>5.758063980116499</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.474467965870814</t>
+          <t>0.889928609792061</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.5800680238165719</t>
+          <t>1.706945796905444</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.0065447590941132</t>
+          <t>0.7735095706155432</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>55.94897304362686</t>
+          <t>30.323632634030773</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>48.505679379380716</t>
+          <t>94.47757544462118</t>
         </is>
       </c>
     </row>
@@ -778,62 +778,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7.282047226851908</t>
+          <t>33.56941366211398</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5.780739425053833</t>
+          <t>22.87756437240393</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.48068711298191</t>
+          <t>4.368006775775588</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9.165257484884245</t>
+          <t>14.525979723390119</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>16.338848404481805</t>
+          <t>131.25690637156202</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.444579617756907</t>
+          <t>0.5527125924949157</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5.4421586637307025</t>
+          <t>4.4220608298296415</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.3423399311427146</t>
+          <t>0.7165686985540617</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.739181741870339</t>
+          <t>0.7856298783301974</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.23466222216815288</t>
+          <t>0.4910510059693771</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>365.598218956435</t>
+          <t>202.28360373884863</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3.6888040000486626</t>
+          <t>6.768406424814756</t>
         </is>
       </c>
     </row>
@@ -845,12 +845,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>22.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -860,47 +860,47 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>134.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>371.0</t>
+          <t>201.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
     </row>
@@ -912,62 +912,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6.6131686357600845</t>
+          <t>8.044497349596059</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7.62239734018649</t>
+          <t>8.202562274773134</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.4226574480958334</t>
+          <t>2.919032565556009</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>27.307821500047357</t>
+          <t>40.1693959298027</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>22.79217823178452</t>
+          <t>31.5054196517122</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.8431778132684613</t>
+          <t>0.9792970408060454</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.569643377269284</t>
+          <t>2.934318166552667</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.7477876008009503</t>
+          <t>1.070019134832567</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.0850594224922185</t>
+          <t>1.132449707924791</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.6511362366835836</t>
+          <t>0.9927783634863282</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>52.937822545582165</t>
+          <t>30.68148104992832</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>13.677610900430235</t>
+          <t>21.52086839264937</t>
         </is>
       </c>
     </row>
@@ -1060,62 +1060,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>27.504632598251042</t>
+          <t>35.714851213603325</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>42.302294460397555</t>
+          <t>69.23941125382822</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.58840038287472</t>
+          <t>4.986058417516113</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>835.7560195898036</t>
+          <t>138.7277871737441</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6.700223963125075</t>
+          <t>13.384358001554144</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4.611679537576552</t>
+          <t>0.8626319879325319</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>37.70111609839508</t>
+          <t>8.031137724550899</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.5876848160435659</t>
+          <t>1.3408328381405128</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.0962669714795505</t>
+          <t>1.3731315993966267</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.5282370106033994</t>
+          <t>0.5442153860218494</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>91.62911334764468</t>
+          <t>153.73806280568633</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>20.992147351008764</t>
+          <t>12.774832015358596</t>
         </is>
       </c>
     </row>
@@ -1127,62 +1127,62 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>881.0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>164.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -1194,62 +1194,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8.475380163948955</t>
+          <t>12.372494521734795</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>23.449059051458335</t>
+          <t>21.431901889371762</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.228909681800784</t>
+          <t>3.0379985061405597</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>167.28567276071715</t>
+          <t>213.69962268145875</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>15.700813387826036</t>
+          <t>18.12170196377285</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.6971703437179</t>
+          <t>1.2379543788136003</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>12.892262247723002</t>
+          <t>6.497073679915053</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.0384649230465117</t>
+          <t>1.4979593930947563</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.7098699510741657</t>
+          <t>4.231076986730177</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.0203262488653233</t>
+          <t>1.0743039676067445</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>18.325942221220053</t>
+          <t>48.244958685216886</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>48.31540386000925</t>
+          <t>41.58669760704523</t>
         </is>
       </c>
     </row>
@@ -1342,62 +1342,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33.47991696780218</t>
+          <t>7.251214273510532</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>22.882917495635226</t>
+          <t>5.685338410094945</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.359185310000406</t>
+          <t>4.480827902662859</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14.319602907141988</t>
+          <t>9.053708720802518</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>131.30922388241504</t>
+          <t>16.33405335481194</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.550869909456332</t>
+          <t>0.4440091772229138</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4.420028218766495</t>
+          <t>5.438322227917308</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.7197105038775428</t>
+          <t>0.3393741915013058</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.7879532258719396</t>
+          <t>0.7402675062849332</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.4940720289090097</t>
+          <t>0.2346415757487003</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>202.28670469771407</t>
+          <t>365.9431060994362</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>6.676981404035892</t>
+          <t>3.677698860169388</t>
         </is>
       </c>
     </row>
@@ -1409,12 +1409,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>134.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>201.0</t>
+          <t>372.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1476,62 +1476,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8.054529424480192</t>
+          <t>6.586829209319877</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>8.199582929401755</t>
+          <t>7.4095662149710995</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.9149789849965027</t>
+          <t>3.424747910847523</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>39.53585016415867</t>
+          <t>26.721181850594114</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>31.4713924212155</t>
+          <t>22.79264168258227</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.9771282328866272</t>
+          <t>0.8424831272733417</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2.9320656604709803</t>
+          <t>3.561449156792119</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.0747063640681511</t>
+          <t>0.7432902050161078</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.1329392440163237</t>
+          <t>1.126546208469699</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.01674806406134</t>
+          <t>0.6552643290961239</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>30.830713392991317</t>
+          <t>52.586186464841724</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>20.863896002642576</t>
+          <t>13.704892229142283</t>
         </is>
       </c>
     </row>
@@ -1624,62 +1624,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>21.3988988988989</t>
+          <t>19.904984423676012</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>23.223973973973973</t>
+          <t>23.10617860851506</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.6956956956956954</t>
+          <t>6.666147455867082</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>445.78628628628627</t>
+          <t>447.6100726895119</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>16.08208208208208</t>
+          <t>16.098130841121495</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.4224224224224224</t>
+          <t>1.4135514018691588</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>9.206456456456456</t>
+          <t>9.210539979231568</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.6966966966966966</t>
+          <t>0.7048286604361371</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.1461461461461462</t>
+          <t>1.2435098650051921</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.6176176176176176</t>
+          <t>1.7341640706126686</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>53.97172172172172</t>
+          <t>53.72689511941849</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>909.006006006006</t>
+          <t>924.4029075804776</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>17.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1741,12 +1741,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>47.5</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>745.0</t>
+          <t>766.0</t>
         </is>
       </c>
     </row>
@@ -1758,62 +1758,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>22.529349977289378</t>
+          <t>19.95358857094464</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21.770222286456587</t>
+          <t>21.30709039201017</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.664324855405024</t>
+          <t>5.659393023519717</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>390.6741925144506</t>
+          <t>393.187204338532</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>26.040783238238575</t>
+          <t>25.881373814481485</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1.8522063616519133</t>
+          <t>1.8370970017327137</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>7.630064628959452</t>
+          <t>7.619321712834192</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.2486625874736625</t>
+          <t>1.2569010113634782</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.756487378426985</t>
+          <t>3.4298937700439858</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5.092825031033969</t>
+          <t>5.882321756254808</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>42.728446862833074</t>
+          <t>42.598778659947655</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>455.53112524835666</t>
+          <t>457.0514247339772</t>
         </is>
       </c>
     </row>
@@ -1906,62 +1906,62 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25.215686274509803</t>
+          <t>27.596104029701397</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>43.72549019607843</t>
+          <t>41.75995735567796</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11.594771241830065</t>
+          <t>6.609860564289121</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>357.6884531590414</t>
+          <t>836.3493654786731</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>12.285403050108933</t>
+          <t>6.609664175963939</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2.4052287581699345</t>
+          <t>4.625898944178957</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>18.583877995642702</t>
+          <t>37.776958973543685</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.6993464052287581</t>
+          <t>0.583750268864969</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>61.09803921568628</t>
+          <t>1.1590090806220834</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.734204793028322</t>
+          <t>0.5312771787414314</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>100.50544662309368</t>
+          <t>91.37758928654927</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>29.38562091503268</t>
+          <t>21.25618389428697</t>
         </is>
       </c>
     </row>
@@ -1973,37 +1973,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>344.0</t>
+          <t>882.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -2013,17 +2013,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>95.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2040,62 +2040,62 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>18.13527281167459</t>
+          <t>8.424956667951374</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>59.428898066624996</t>
+          <t>22.909761566879418</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>17.32670986139239</t>
+          <t>4.283013518051386</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>261.13629046500813</t>
+          <t>168.13791911197407</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>22.455359356629586</t>
+          <t>15.669228126337979</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.365615826255409</t>
+          <t>2.697589695676837</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>12.938561093671023</t>
+          <t>12.89724445561392</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.0831546397838743</t>
+          <t>1.0345913484459113</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>32.964779125939735</t>
+          <t>2.595384389789606</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>7.835950471543475</t>
+          <t>1.0319368466593075</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>47.64352782650311</t>
+          <t>18.09161798306015</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>82.91264722544065</t>
+          <t>49.23292776822658</t>
         </is>
       </c>
     </row>

</xml_diff>